<commit_message>
SQL-Agents: agentes, orquestador, experimentos e informe de tesis (2026-05-30)
</commit_message>
<xml_diff>
--- a/informe/SQL_Agents_v3.xlsx
+++ b/informe/SQL_Agents_v3.xlsx
@@ -34,8 +34,8 @@
     <sheet name="Fase 2 - AS" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="Fase 3 - Orch MySQL" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="Fase 3 - Orch Postgres" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Fase 4 - Orch MySQL" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Fase 4 - Orch Postgres" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Fase 4_1 - Orch MySQL" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Fase 4_1 - Orch Postgres" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="Fase 3_2 - Orch MySQL" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="Fase 3_2 - Orch Postgres" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="Fase 4_2 - Orch MySQL" sheetId="33" state="visible" r:id="rId33"/>
@@ -67,7 +67,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -133,6 +133,15 @@
     <font>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="13">
@@ -283,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -372,6 +381,26 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10712,310 +10741,224 @@
   <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="40" customWidth="1" style="23" min="1" max="3"/>
+    <col width="22" customWidth="1" style="23" min="1" max="3"/>
+    <col width="22" customWidth="1" style="23" min="2" max="2"/>
+    <col width="22" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="23">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="23">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>PARÁMETRO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>FASE 3 (winner)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>FASE 4 (robustez)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C3" s="2" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>FASE 3 Exp1 (ganador)</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>FASE 4 Exp1 (robustez)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="23">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B2" s="32" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash</t>
+        </is>
+      </c>
+      <c r="C2" s="32" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="23">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Temperatura</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C3" s="34" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" s="23">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Faithfulness</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>0.857</v>
-      </c>
-      <c r="C4" s="3" t="n">
+      <c r="B4" s="35" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="C4" s="35" t="n">
         <v>0.821</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="5" ht="20" customHeight="1" s="23">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Groundedness</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>0.948</v>
-      </c>
-      <c r="C5" s="3" t="n">
+      <c r="B5" s="33" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="C5" s="33" t="n">
         <v>0.9320000000000001</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6" ht="20" customHeight="1" s="23">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Correctness</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="35" t="n">
         <v>0.991</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="35" t="n">
         <v>0.791</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7" ht="20" customHeight="1" s="23">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>ROUGE-L_SQL</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="33" t="n">
         <v>0.591</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="33" t="n">
         <v>0.526</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>WACS</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="3" t="n">
-        <v>0.656</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="8" ht="20" customHeight="1" s="23">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Brier</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>0.0051</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>0.09719999999999999</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="B8" s="32" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="C8" s="35" t="n">
+        <v>0.097</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="23">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>ECE</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="C10" s="3" t="n">
+      <c r="B9" s="33" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="C9" s="33" t="n">
         <v>0.034</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="10" ht="20" customHeight="1" s="23">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>combined_score</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>2.7435</v>
-      </c>
-      <c r="C11" s="3" t="n">
+      <c r="B10" s="35" t="n">
+        <v>2.705</v>
+      </c>
+      <c r="C10" s="35" t="n">
         <v>2.413</v>
       </c>
     </row>
+    <row r="11" ht="20" customHeight="1" s="23">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>n_evaluados</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>30</v>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>n_cases</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
     </row>
+    <row r="13">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>Nota: Exp1 usa gemini-2.5-flash (corrida original sin correcciones de prompts ni normalización de JOINs).</t>
+        </is>
+      </c>
+    </row>
     <row r="14" ht="27.6" customHeight="1" s="23">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Nota: phase_4 original (2026-05-25). Gap: alternative_vocabulary punto debil (2.332).</t>
-        </is>
-      </c>
-    </row>
+      <c r="A14" s="2" t="n"/>
+    </row>
+    <row r="15"/>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>-- PREGUNTAS DE PRUEBA (10 casos) --</t>
-        </is>
-      </c>
+      <c r="A16" s="37" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Pregunta Usuario</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>SQL Esperado</t>
-        </is>
-      </c>
+      <c r="A17" s="38" t="n"/>
+      <c r="B17" s="38" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>How many singers are there?</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>SELECT COUNT(*) FROM singer</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
     </row>
     <row r="19" ht="27.6" customHeight="1" s="23">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>How many concerts took place in 2014?</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>SELECT COUNT(*) FROM concert WHERE year=2014</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
     </row>
     <row r="20" ht="27.6" customHeight="1" s="23">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>What are the names and capacities of all stadiums?</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>SELECT name, capacity FROM stadium</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
     </row>
     <row r="21" ht="27.6" customHeight="1" s="23">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>List the names of singers from France.</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>SELECT name FROM singer WHERE country='France'</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
     </row>
     <row r="22" ht="27.6" customHeight="1" s="23">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>How many singers performed in each concert?</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>SELECT concert_id, COUNT(singer_id) FROM singer_in_concert GROUP BY concert_id</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>What is the average age of all singers?</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>SELECT AVG(age) FROM singer</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
     </row>
     <row r="24" ht="27.6" customHeight="1" s="23">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Which stadiums have hosted more than 2 concerts?</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>SELECT stadium_id, COUNT(*) FROM concert GROUP BY stadium_id HAVING COUNT(*)&gt;2</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
     </row>
     <row r="25" ht="41.4" customHeight="1" s="23">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>List all concerts held at stadiums with capacity above 5000.</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>SELECT c.* FROM concert c JOIN stadium s ON c.stadium_id=s.stadium_id WHERE s.capacity&gt;5000</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
     </row>
     <row r="26" ht="27.6" customHeight="1" s="23">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>What is the name of the youngest singer?</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>SELECT name FROM singer ORDER BY age ASC LIMIT 1</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
     </row>
     <row r="27" ht="41.4" customHeight="1" s="23">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Show all concerts with their stadium names and themes.</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>SELECT c.concert_name, s.name, c.theme FROM concert c JOIN stadium s ON c.stadium_id=s.stadium_id</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11575,354 +11518,241 @@
   <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="40" customWidth="1" style="23" min="1" max="3"/>
+    <col width="22" customWidth="1" style="23" min="1" max="3"/>
+    <col width="22" customWidth="1" style="23" min="2" max="2"/>
+    <col width="22" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="23">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="23">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>PARÁMETRO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>FASE 3 (winner)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>FASE 4 (robustez)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>claude-haiku-4-5</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C3" s="2" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>FASE 3 Exp1 (ganador)</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>FASE 4 Exp1 (robustez)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="23">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B2" s="32" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash</t>
+        </is>
+      </c>
+      <c r="C2" s="32" t="inlineStr">
+        <is>
+          <t>gemini-2.5-flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="23">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Temperatura</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="34" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" s="23">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Faithfulness</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.786</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="B4" s="35" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="C4" s="35" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" s="23">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Groundedness</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B5" s="33" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="C5" s="33" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" s="23">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Correctness</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="35" t="n">
         <v>0.8</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="35" t="n">
         <v>0.9</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7" ht="20" customHeight="1" s="23">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>ROUGE-L_SQL</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>0.575</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>0.524</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>WACS</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="B7" s="33" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>0.485</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" s="23">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Brier</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>0.0045</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>0.09089999999999999</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="B8" s="32" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="23">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>ECE</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>0.0356</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="B9" s="33" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>0.261</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" s="23">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>combined_score</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>2.5537</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>2.4952</v>
+      <c r="B10" s="35" t="n">
+        <v>2.253</v>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>2.098</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" s="23">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>n_evaluados</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>n_cases</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>Nota: Exp1 usa gemini-2.5-flash (corrida original sin correcciones de prompts ni normalización de JOINs).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Desglose por variante de paráfrasis (Fase 4)</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="inlineStr">
-        <is>
-          <t>Combined Score</t>
-        </is>
-      </c>
+      <c r="A14" s="37" t="n"/>
+      <c r="B14" s="37" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>informal</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>2.575</v>
-      </c>
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>open_rephrased</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>2.539</v>
-      </c>
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>alternative_vocabulary</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>2.371</v>
-      </c>
-    </row>
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="3" t="n"/>
+    </row>
+    <row r="18"/>
     <row r="19" ht="55.2" customHeight="1" s="23">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Nota: phase_4_2 claude-haiku-4-5 T=0.3 (ganador phase_3_2). Bug1+Bug2+Bug3 corregidos. ROUGE 0.70. Sin fixes con gpt-4o: 2.262. Con fixes gpt-4o: 2.504.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A19" s="2" t="n"/>
+    </row>
+    <row r="20"/>
     <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>-- PREGUNTAS DE PRUEBA (10 casos) --</t>
-        </is>
-      </c>
+      <c r="A21" s="37" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Pregunta Usuario</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>SQL Esperado</t>
-        </is>
-      </c>
+      <c r="A22" s="38" t="n"/>
+      <c r="B22" s="38" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>How many singers are there?</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>SELECT COUNT(*) FROM singer</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
     </row>
     <row r="24" ht="27.6" customHeight="1" s="23">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>How many concerts took place in 2014?</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>SELECT COUNT(*) FROM concert WHERE year=2014</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
     </row>
     <row r="25" ht="27.6" customHeight="1" s="23">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>What are the names and capacities of all stadiums?</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>SELECT name, capacity FROM stadium</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
     </row>
     <row r="26" ht="27.6" customHeight="1" s="23">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>List the names of singers from France.</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>SELECT name FROM singer WHERE country='France'</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
     </row>
     <row r="27" ht="27.6" customHeight="1" s="23">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>How many singers performed in each concert?</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>SELECT concert_id, COUNT(singer_id) FROM singer_in_concert GROUP BY concert_id</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>What is the average age of all singers?</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>SELECT AVG(age) FROM singer</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
     </row>
     <row r="29" ht="27.6" customHeight="1" s="23">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Which stadiums have hosted more than 2 concerts?</t>
-        </is>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>SELECT stadium_id, COUNT(*) FROM concert GROUP BY stadium_id HAVING COUNT(*)&gt;2</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
     </row>
     <row r="30" ht="41.4" customHeight="1" s="23">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>List all concerts held at stadiums with capacity above 5000.</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>SELECT c.* FROM concert c JOIN stadium s ON c.stadium_id=s.stadium_id WHERE s.capacity&gt;5000</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
     </row>
     <row r="31" ht="27.6" customHeight="1" s="23">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>What is the name of the youngest singer?</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>SELECT name FROM singer ORDER BY age ASC LIMIT 1</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
     </row>
     <row r="32" ht="41.4" customHeight="1" s="23">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Show all concerts with their stadium names and themes.</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>SELECT c.concert_name, s.name, c.theme FROM concert c JOIN stadium s ON c.stadium_id=s.stadium_id</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>